<commit_message>
update file and add readme
</commit_message>
<xml_diff>
--- a/02_Test_Case/Register/test_register.xlsx
+++ b/02_Test_Case/Register/test_register.xlsx
@@ -8,12 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ucupcode\QA\Tool-Shop\02_Test_Case\Register\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{267F055B-4EE8-49BC-BA8B-643CB4580C0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9BC0D1F-1CB5-423D-AF4D-569DB4FF115E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{A484E914-C329-4284-B44D-62BA54F2470F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="1" xr2:uid="{A484E914-C329-4284-B44D-62BA54F2470F}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Acceptance Criteria" sheetId="3" r:id="rId1"/>
+    <sheet name="Test Case" sheetId="4" r:id="rId2"/>
+    <sheet name="Test_Case" sheetId="1" r:id="rId3"/>
+    <sheet name="Summary" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="321">
   <si>
     <t>TEST CASE - REGISTER</t>
   </si>
@@ -237,9 +240,6 @@
   </si>
   <si>
     <t>Register dengan password tanpa simbol</t>
-  </si>
-  <si>
-    <t>Register dengan invalid format phone</t>
   </si>
   <si>
     <t>Register dengan mengisi date of birth dimasa mendatang</t>
@@ -849,12 +849,6 @@
 Password: Customer@41</t>
   </si>
   <si>
-    <t>Register dengan membuat password dengan panjang karakter 5</t>
-  </si>
-  <si>
-    <t>Register dengan membuat password dengan panjang karakter 6</t>
-  </si>
-  <si>
     <t>First name: yuyaa
 Last name: testing
 Date of Birth: 2000-04-21
@@ -992,9 +986,6 @@
 Password: Custom41&gt;&lt;</t>
   </si>
   <si>
-    <t xml:space="preserve">User berhasil melakukan register dan diarahkan menuju </t>
-  </si>
-  <si>
     <t>Memastikan kolom alamat terisi secara otomatis setelah memasukkan country, postal code, dan house number</t>
   </si>
   <si>
@@ -1008,13 +999,572 @@
   </si>
   <si>
     <t>Memastikan kolom alamat berubah ketika country diganti</t>
+  </si>
+  <si>
+    <t>TC_REG_037</t>
+  </si>
+  <si>
+    <t>TC_REG_038</t>
+  </si>
+  <si>
+    <t>TC_REG_039</t>
+  </si>
+  <si>
+    <t>TC_REG_040</t>
+  </si>
+  <si>
+    <t>Register dengan umur 17 tahun</t>
+  </si>
+  <si>
+    <t>Register dengan umur 18 tahun</t>
+  </si>
+  <si>
+    <t>Register dengan umur 75 tahun</t>
+  </si>
+  <si>
+    <t>Register dengan umur 76 tahun</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa semua data harus diisi</t>
+  </si>
+  <si>
+    <t>1. Masuk ke halaman web
+2. Masuk ke form sign in
+3. Klik link menuju registrasi
+4. Isi form dengan data valid
+5. Isi field country, postal code, dan house number
+6. Alamat lain terisi secara otomatis
+7. Klik tombol registrasi</t>
+  </si>
+  <si>
+    <t>1. Masuk ke halaman web
+2. Masuk ke form sign in
+3. Klik link menuju registrasi
+4. Isi form dengan data valid
+5. Isi field country, postal code, dan house number
+6. Alamat lain terisi secara otomatis
+7. Mengubah isi dari alamat yang telah terisi 
+8. Klik tombol registrasi</t>
+  </si>
+  <si>
+    <t>1. Masuk ke halaman web
+2. Masuk ke form sign in
+3. Klik link menuju registrasi
+4. Isi form dengan data valid
+5. Isi field country, postal code, dan house number
+6. Alamat lain terisi secara otomatis
+7. Ubah country untuk update alamat lainnya
+8. Klik tombol registrasi</t>
+  </si>
+  <si>
+    <t>1. Masuk ke halaman web
+2. Masuk ke form sign in
+3. Klik link menuju registrasi
+4. Isi form dengan data valid
+5. Isi field date of birth dengan tanggal yang sama dengan umur 17 tahun
+6. Klik tombol registrasi</t>
+  </si>
+  <si>
+    <t>1. Masuk ke halaman web
+2. Masuk ke form sign in
+3. Klik link menuju registrasi
+4. Isi form dengan data valid
+5. Isi field date of birth dengan tanggal yang sama dengan umur 18 tahun
+6. Klik tombol registrasi</t>
+  </si>
+  <si>
+    <t>1. Masuk ke halaman web
+2. Masuk ke form sign in
+3. Klik link menuju registrasi
+4. Isi form dengan data valid
+5. Isi field date of birth dengan tanggal yang sama dengan umur 75 tahun
+6. Klik tombol registrasi</t>
+  </si>
+  <si>
+    <t>1. Masuk ke halaman web
+2. Masuk ke form sign in
+3. Klik link menuju registrasi
+4. Isi form dengan data valid
+5. Isi field date of birth dengan tanggal yang sama dengan umur 76 tahun
+6. Klik tombol registrasi</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa first name wajib diisi</t>
+  </si>
+  <si>
+    <t>Medapatkan pesan eror bahwa last name wajib diisi</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa date of birth wajib diisi</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa country wajib diisi</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa postal code wajb diisi</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa house number wajib diisi</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa street waji diisi</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa city wajib diisi</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa state wajib diisi</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa phone wajib diisi</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa email address wajib diisi</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa password wajib diisi dan minimal terdiri dari 8 karakter</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa first name dan last name wajib diisi</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa email address dan password wajib diisi</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa phone tidak boleh hanya mengandung 1 digit</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa phone tidak boleh melewati batas maksimum</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa email address invalid format</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa password minimal terdiri dari 8 karakter</t>
+  </si>
+  <si>
+    <t>Password valid, user dapat lanjut melakukan registrasi</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa password harus mengandung uppercase, angka, dan simbol spesial</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa password harus mengandung uppercase</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa password harus mengandung lowercase</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa password setidaknya mengandung satu angka</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa password setidaknya mengandung satu simbol spesial</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa password tidak boleh mengandung invalid character</t>
+  </si>
+  <si>
+    <t>Alamat lain terisi secara otomatis</t>
+  </si>
+  <si>
+    <t>User dapat mengubah isi alamat yang terisi secara otomatis dan perubahan berhasil disimpan</t>
+  </si>
+  <si>
+    <t>Alamat lain akan berubah secara otomatis setelah country diganti</t>
+  </si>
+  <si>
+    <t>User berhasil melakukan register dan diarahkan menuju form sign in</t>
+  </si>
+  <si>
+    <t>User berhasil melakukan registrasi dan diarahkan menuju form sign in</t>
+  </si>
+  <si>
+    <t>User mendapatkan pesan eror bahwa semua field data wajib diisi</t>
+  </si>
+  <si>
+    <t>User mendapatkan pesan eror "First name is required"</t>
+  </si>
+  <si>
+    <t>User mendapatkan pesan eror "Last name is required"</t>
+  </si>
+  <si>
+    <t>User mendapatkan pesan eror "Please enter a valid date in YYYY-MM-DD format.
+Date of Birth is required"</t>
+  </si>
+  <si>
+    <t>User mendapatkan pesan eror "Country is required"</t>
+  </si>
+  <si>
+    <t>User mendapatkan pesan eror "House number is required"</t>
+  </si>
+  <si>
+    <t>User mendapatkan pesan eror "City is required"</t>
+  </si>
+  <si>
+    <t>User mendapatkan pesan eror "State is required"</t>
+  </si>
+  <si>
+    <t>User mendapatkan pesan eror "Phone is required"</t>
+  </si>
+  <si>
+    <t>User mendapatkan pesan eror "Postcode is required"</t>
+  </si>
+  <si>
+    <t>User mendapatkan pesan eror "Street is required"</t>
+  </si>
+  <si>
+    <t>User mendapatkan pesan eror "Email is required"</t>
+  </si>
+  <si>
+    <t>User mendapatkan pesan eror "Password is required
+Password must be minimal 6 characters long.
+Password can not include invalid characters."</t>
+  </si>
+  <si>
+    <t>User mendapatkan pesan eror "First name is required" dan "Last name is required"</t>
+  </si>
+  <si>
+    <t>Sistem menampilkan pesan "Email is required" dan "Password is required
+Password must be minimal 6 characters long.
+Password can not include invalid characters."</t>
+  </si>
+  <si>
+    <t>User tidak dapat melakukan registrasi dengan Date of Birth di masa mendatang.</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Sistem menampilkan pesan "Customer must be 18 years old."</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Sistem menampilkan pesan "Only numbers are allowed."</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa phone hanya boleh  berupa angka</t>
+  </si>
+  <si>
+    <t>Sistem menerima phone hanya 1 digit</t>
+  </si>
+  <si>
+    <t>low</t>
+  </si>
+  <si>
+    <t>Sistem menerima banyak digit</t>
+  </si>
+  <si>
+    <t>Berhasil login dan diarahkan menuju form sign in</t>
+  </si>
+  <si>
+    <t>Berhasil melakukan registrasi dan diarahkan menuju form login</t>
+  </si>
+  <si>
+    <t>Sistem menampilkan pesan "A customer with this email address already exists.
+The given password has appeared in a data leak. Please choose a different password."</t>
+  </si>
+  <si>
+    <t>Sistem menolak dan memberikan pesan eror pada user bahwa akun sudah pernah digunakan</t>
+  </si>
+  <si>
+    <t>Sistem menampilkan pesan "Email format is invalid"</t>
+  </si>
+  <si>
+    <t>Sistem menampilkan pesan "Password must be minimal 6 characters long."</t>
+  </si>
+  <si>
+    <t>Sistem menampilkan pesan "Password can not include invalid characters."</t>
+  </si>
+  <si>
+    <t>Sistem menerima password yang berisi invalid character</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Sistem menampilkan alamat lain secara otomatis</t>
+  </si>
+  <si>
+    <t>Sistem menerima perubahan yang dilakukan pada alamat yang sudah diisi otomatis</t>
+  </si>
+  <si>
+    <t>Sistem mengubah alamat ketika country diganti</t>
+  </si>
+  <si>
+    <t>Mendapatkan pesan eror bahwa umur customer harus diatas 18 tahun</t>
+  </si>
+  <si>
+    <t>Sistem menerima dan user dapat melanjutkan registrasi</t>
+  </si>
+  <si>
+    <t>Sistem menerima input dan user berhasil melakukan registrasi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sistem menerima input dan user berhasil melakukan registrasi </t>
+  </si>
+  <si>
+    <t>Sistem menerima input dan user diarahkan menuju halaman My Account</t>
+  </si>
+  <si>
+    <t>Sistem menolak input dan memberikan pesan validasi bahwa umur tidak boleh melewati 75 tahun</t>
+  </si>
+  <si>
+    <t>Feature</t>
+  </si>
+  <si>
+    <t>Total Scenario Executed</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Execution Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">: </t>
+  </si>
+  <si>
+    <t>Registrasi</t>
+  </si>
+  <si>
+    <t>:</t>
+  </si>
+  <si>
+    <t>Summary Report</t>
+  </si>
+  <si>
+    <t>Acceptance Criteria</t>
+  </si>
+  <si>
+    <t>AC_ID</t>
+  </si>
+  <si>
+    <t>AC_001</t>
+  </si>
+  <si>
+    <t>AC_002</t>
+  </si>
+  <si>
+    <t>AC_003</t>
+  </si>
+  <si>
+    <t>AC_004</t>
+  </si>
+  <si>
+    <t>Email harus bersifat unik dan dengan format yang valid</t>
+  </si>
+  <si>
+    <t>Semua mandatory field wajib diisi</t>
+  </si>
+  <si>
+    <t>Field name, address, dan phone harus diisi berdasarkan aturan validasi dan panjang maksimal</t>
+  </si>
+  <si>
+    <t>AC_005</t>
+  </si>
+  <si>
+    <t>AC_006</t>
+  </si>
+  <si>
+    <t>Password harus terdiri dari minimal 8 karakter</t>
+  </si>
+  <si>
+    <t>Password harus mengandung huruf besar, huruf kecil, angka, dan simbol, belum pernah digunakan sebelumnya, serta harus sama dengan password konfirmasi</t>
+  </si>
+  <si>
+    <t>Test Case</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Pre-Conditions</t>
+  </si>
+  <si>
+    <t>Test Steps</t>
+  </si>
+  <si>
+    <t>AC References</t>
+  </si>
+  <si>
+    <t>Register dengan menggunakan data valid</t>
+  </si>
+  <si>
+    <t>User berada pada halaman registrasi</t>
+  </si>
+  <si>
+    <t>Sistem menerima input data dan user diarahkan menuju form sign in</t>
+  </si>
+  <si>
+    <t>Register dengan mengosongkan semua field</t>
+  </si>
+  <si>
+    <t>Sistem menolak registasi dan memberikan pesan validasi bahwa tiap field wajib diisi</t>
+  </si>
+  <si>
+    <t>Sistem memberikan pesan validasi bahwa tiap field wajib diisi</t>
+  </si>
+  <si>
+    <t>Register dengan mengosongkan field First name</t>
+  </si>
+  <si>
+    <t>Register dengan mengosongkan field Last name</t>
+  </si>
+  <si>
+    <t>Register dengan mengosongkan field Date of Birth</t>
+  </si>
+  <si>
+    <t>Register dengan mengosongkan field Country</t>
+  </si>
+  <si>
+    <t>Register dengan mengosongkan field Postal code</t>
+  </si>
+  <si>
+    <t>Register dengan mengosongkan field Street</t>
+  </si>
+  <si>
+    <t>Register dengan mengosongkan field House number</t>
+  </si>
+  <si>
+    <t>Register dengan mengosongkan field State</t>
+  </si>
+  <si>
+    <t>Register dengan mengosongkan field City</t>
+  </si>
+  <si>
+    <t>Register dengan mengosongkan field Phone</t>
+  </si>
+  <si>
+    <t>Register dengan mengosongkan field Email</t>
+  </si>
+  <si>
+    <t>Register dengan mengosongkan field Password</t>
+  </si>
+  <si>
+    <t>Register dengan mengosongkan field First name dan Last name</t>
+  </si>
+  <si>
+    <t>Register dengan mengosongkan field Email dan Password</t>
+  </si>
+  <si>
+    <t>Umur harus berada diantara 18 dan 75 tahun</t>
+  </si>
+  <si>
+    <t>Register dengan mengisi field Date of Birth dengan tanggal dimasa mendatang</t>
+  </si>
+  <si>
+    <t>Register dengan mengisi Date of Birth yang setara dengan umur 17 tahun</t>
+  </si>
+  <si>
+    <t>Register dengan mengisi Date of Birth yang setara dengan umur 18 tahun</t>
+  </si>
+  <si>
+    <t>Register dengan mengisi Date of Birth yang setara dengan umur 75 tahun</t>
+  </si>
+  <si>
+    <t>Register dengan mengisi Date of Birth yang setara dengan umur 76 tahun</t>
+  </si>
+  <si>
+    <t>Mengisi field Date of Birth dengan format  YYYY/MM/DD</t>
+  </si>
+  <si>
+    <t>Exploratory Test</t>
+  </si>
+  <si>
+    <t>Memastikan seluruh field alamat terisi secara otomatis setelah mengisi field Country, Postal code, dan House Number</t>
+  </si>
+  <si>
+    <t>Mengubah isi alamat setelah terisi secara otomatis</t>
+  </si>
+  <si>
+    <t>Memastikan seluruh field alamat berubah ketika isi field country diganti</t>
+  </si>
+  <si>
+    <t>Mengisi field Phone dengan huruf</t>
+  </si>
+  <si>
+    <t>Mengisi field phone dengan simbol</t>
+  </si>
+  <si>
+    <t>Mengisi field Phone hanya dengan 1 digit</t>
+  </si>
+  <si>
+    <t>Mengisi field Phone lebih dari 15 digit</t>
+  </si>
+  <si>
+    <t>Register dengan email yang belum teregistrasi</t>
+  </si>
+  <si>
+    <t>Register dengan email yang telah teregistrasi</t>
+  </si>
+  <si>
+    <t>Register dengan panjang password 7 karakter</t>
+  </si>
+  <si>
+    <t>Register dengan panjang password 8 karakter</t>
+  </si>
+  <si>
+    <t>Register dengan panjang password 9 karakter</t>
+  </si>
+  <si>
+    <t>Mengisi field password hanya dengan huruf</t>
+  </si>
+  <si>
+    <t>Mengisi field password tanpa huruf besar</t>
+  </si>
+  <si>
+    <t>Mengisi field password tanpa huruf kecil</t>
+  </si>
+  <si>
+    <t>Mengisi field password hanya dengan angka</t>
+  </si>
+  <si>
+    <t>Mengisi field password tanpa angka</t>
+  </si>
+  <si>
+    <t>TC_REG_041</t>
+  </si>
+  <si>
+    <t>TC_REG_042</t>
+  </si>
+  <si>
+    <t>Mengisi field password hanya dengan simbol</t>
+  </si>
+  <si>
+    <t>Mengisi field password tanpa simbol</t>
+  </si>
+  <si>
+    <t>TC_REG_043</t>
+  </si>
+  <si>
+    <t>TC_REG_044</t>
+  </si>
+  <si>
+    <t>TC_REG_045</t>
+  </si>
+  <si>
+    <t>Mengisi field password dengan password yang belum pernah digunakan</t>
+  </si>
+  <si>
+    <t>Mengisi field password dengan password yang sudah pernah digunakan</t>
+  </si>
+  <si>
+    <t>Mengisi field password sama dengan confirm password</t>
+  </si>
+  <si>
+    <t>Column1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1058,6 +1608,14 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Aptos Display"/>
+      <family val="2"/>
+      <scheme val="major"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1105,7 +1663,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1126,12 +1684,23 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Title" xfId="1" builtinId="15"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="34">
     <dxf>
       <fill>
         <patternFill>
@@ -1149,44 +1718,50 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B050"/>
+          <bgColor rgb="FF15DF0B"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF2929"/>
+          <bgColor rgb="FFFF4A37"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B050"/>
+          <bgColor rgb="FF15DF0B"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF2929"/>
+          <bgColor rgb="FFFF4A37"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B050"/>
+          <bgColor rgb="FF15DF0B"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF2929"/>
+          <bgColor rgb="FFFF4A37"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1196,6 +1771,28 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1235,28 +1832,47 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-      </border>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFF4A37"/>
+      <color rgb="FF15DF0B"/>
       <color rgb="FFFF2929"/>
     </mruColors>
   </colors>
@@ -1271,164 +1887,52 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>1114425</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>962025</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>152400</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>323850</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="TextBox 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E116225D-AAE9-85C0-91E8-9823C23F8B51}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6600825" y="4914900"/>
-          <a:ext cx="3800475" cy="2219325"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:schemeClr val="lt1">
-              <a:shade val="50000"/>
-            </a:schemeClr>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100"/>
-            <a:t>First name: yuyaa</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100"/>
-            <a:t>Last name: testing</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100"/>
-            <a:t>Date of Birth: 2000-04-21</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100"/>
-            <a:t>Country: Indonesia</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100"/>
-            <a:t>Postal Code: 22543</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100"/>
-            <a:t>House</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t> Number: 12</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t>Street: Jl. Merpati</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t>City: Bandung</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t>State: Jawa Barat</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t>Phone: 081234564321</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t>Email: customertester@gmail.com</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t>Password: Customer@41</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8805D3A0-FDED-4771-9909-013818D3A66A}" name="Table2" displayName="Table2" ref="A3:C9" totalsRowShown="0">
+  <autoFilter ref="A3:C9" xr:uid="{8805D3A0-FDED-4771-9909-013818D3A66A}"/>
+  <tableColumns count="3">
+    <tableColumn id="3" xr3:uid="{CCBF4BAD-7A47-4E64-A33C-10EB349C351E}" name="Column1"/>
+    <tableColumn id="1" xr3:uid="{577634A3-7EA6-4D6A-A0F3-B2E6B3CA18DA}" name="AC_ID"/>
+    <tableColumn id="2" xr3:uid="{A88AD446-0555-4F57-A883-82A8FAE740F0}" name="Acceptance Criteria"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{81A745C3-79A0-45D2-95F5-8204D4B2F75C}" name="Table1" displayName="Table1" ref="A3:I39" totalsRowShown="0" headerRowDxfId="11" dataDxfId="19" tableBorderDxfId="18">
-  <autoFilter ref="A3:I39" xr:uid="{81A745C3-79A0-45D2-95F5-8204D4B2F75C}"/>
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{280ADF9C-15E8-46ED-9AC3-0E1DA28D7AFA}" name="Table3" displayName="Table3" ref="A3:L48" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
+  <autoFilter ref="A3:L48" xr:uid="{280ADF9C-15E8-46ED-9AC3-0E1DA28D7AFA}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{2961E5F0-50D5-456A-966B-3296F1DE5F27}" name="No" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{405819EF-CA2E-4FD8-BA13-2235D9ED1DAD}" name="Test Case ID" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{1564669D-18D9-4642-B9B7-3EC5553573CF}" name="Test Case" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{4A190C8C-C094-4C48-AA6E-98E8EFC4B1A0}" name="Pre-Conditions" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{C6683DEA-5756-400B-8CA2-E2EDE1F731DE}" name="Test Steps" dataDxfId="27"/>
+    <tableColumn id="6" xr3:uid="{A5C8FC0E-6FEB-4A01-9F73-4C2FF9C03534}" name="Test Data" dataDxfId="26"/>
+    <tableColumn id="7" xr3:uid="{7C519673-CEC3-42BF-B787-00204C720E44}" name="Expected Result" dataDxfId="25"/>
+    <tableColumn id="8" xr3:uid="{BDC6C98E-7F98-48CB-B54D-27580EC4D707}" name="Actual Result" dataDxfId="24"/>
+    <tableColumn id="9" xr3:uid="{762C8823-2514-4292-8FB1-BF2A3C22FFFA}" name="Status" dataDxfId="23"/>
+    <tableColumn id="12" xr3:uid="{A21FB4B7-4C6E-4B24-A6D3-AA02D1038E77}" name="AC References" dataDxfId="22"/>
+    <tableColumn id="10" xr3:uid="{7BE6C741-7928-4331-ABE0-AA3A8DF91BE9}" name="Severity" dataDxfId="21"/>
+    <tableColumn id="11" xr3:uid="{9FE0EA18-785F-4A85-9D1F-CECC4677CB09}" name="Priority" dataDxfId="20"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{81A745C3-79A0-45D2-95F5-8204D4B2F75C}" name="Table1" displayName="Table1" ref="A3:I43" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18" tableBorderDxfId="17">
+  <autoFilter ref="A3:I43" xr:uid="{81A745C3-79A0-45D2-95F5-8204D4B2F75C}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{A335D1B6-EB44-4FB1-8FC5-F5D61E7FB62F}" name="Test Case ID" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{288F05E7-ACF6-46C5-A6AD-9B4D9DDF4620}" name="Scenario" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{9DC90E0A-1CAB-4E79-8F0D-6353C78C6473}" name="Steps" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{8DADA52D-3A51-40E1-BDF5-81467F53078E}" name="Test Data" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{4815E016-50BA-4DC6-93B0-A3CE5A1BE917}" name="Expected Result" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{04ED4A9F-408A-4A25-96D4-BCF0B8042A38}" name="Actual Result" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{F9C79A6F-D08E-46E4-A85F-5534C7448A19}" name="Status" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{A335D1B6-EB44-4FB1-8FC5-F5D61E7FB62F}" name="Test Case ID" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{288F05E7-ACF6-46C5-A6AD-9B4D9DDF4620}" name="Scenario" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{9DC90E0A-1CAB-4E79-8F0D-6353C78C6473}" name="Steps" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{8DADA52D-3A51-40E1-BDF5-81467F53078E}" name="Test Data" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{4815E016-50BA-4DC6-93B0-A3CE5A1BE917}" name="Expected Result" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{04ED4A9F-408A-4A25-96D4-BCF0B8042A38}" name="Actual Result" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{F9C79A6F-D08E-46E4-A85F-5534C7448A19}" name="Status" dataDxfId="10"/>
     <tableColumn id="8" xr3:uid="{392653D9-B4F4-4FF4-A33C-6C76C79B54A0}" name="Severity" dataDxfId="9"/>
-    <tableColumn id="9" xr3:uid="{5EE02DF5-D969-476E-8BF9-DFD01CD4B6B9}" name="Priority" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{5EE02DF5-D969-476E-8BF9-DFD01CD4B6B9}" name="Priority" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1750,16 +2254,1183 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F4E50C2-6104-4A80-8524-967FEE4AD08E}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8.5703125" customWidth="1"/>
+    <col min="2" max="2" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="147.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="24" x14ac:dyDescent="0.4">
+      <c r="A1" s="10" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>320</v>
+      </c>
+      <c r="B3" t="s">
+        <v>248</v>
+      </c>
+      <c r="C3" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>249</v>
+      </c>
+      <c r="C4" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>250</v>
+      </c>
+      <c r="C5" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C6" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>252</v>
+      </c>
+      <c r="C7" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>256</v>
+      </c>
+      <c r="C8" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>257</v>
+      </c>
+      <c r="C9" t="s">
+        <v>259</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6EDBC65-0C5F-4A06-8710-D45CCBBE14A7}">
+  <dimension ref="A1:L48"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="4" max="4" width="28.28515625" customWidth="1"/>
+    <col min="5" max="5" width="26.140625" customWidth="1"/>
+    <col min="6" max="6" width="33.140625" customWidth="1"/>
+    <col min="7" max="8" width="27.7109375" customWidth="1"/>
+    <col min="10" max="10" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="24" x14ac:dyDescent="0.4">
+      <c r="A1" s="10" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>263</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="I3" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="L3" s="12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="180" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+    </row>
+    <row r="5" spans="1:12" ht="105" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+    </row>
+    <row r="6" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+    </row>
+    <row r="7" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>4</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+    </row>
+    <row r="8" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+    </row>
+    <row r="9" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>6</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+    </row>
+    <row r="10" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>7</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+    </row>
+    <row r="11" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>8</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+    </row>
+    <row r="12" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>9</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+    </row>
+    <row r="13" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>10</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+    </row>
+    <row r="14" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>11</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+    </row>
+    <row r="15" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <v>12</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+    </row>
+    <row r="16" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>13</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+    </row>
+    <row r="17" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>14</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K17" s="2"/>
+      <c r="L17" s="2"/>
+    </row>
+    <row r="18" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <v>15</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
+    </row>
+    <row r="19" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
+        <v>16</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="7"/>
+      <c r="J19" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K19" s="2"/>
+      <c r="L19" s="2"/>
+    </row>
+    <row r="20" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
+        <v>17</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="7"/>
+      <c r="J20" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
+    </row>
+    <row r="21" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
+        <v>18</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2"/>
+    </row>
+    <row r="22" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A22" s="2">
+        <v>19</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="K22" s="2"/>
+      <c r="L22" s="2"/>
+    </row>
+    <row r="23" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" s="2">
+        <v>20</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="7"/>
+      <c r="J23" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="K23" s="2"/>
+      <c r="L23" s="2"/>
+    </row>
+    <row r="24" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A24" s="2">
+        <v>21</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="7"/>
+      <c r="J24" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
+    </row>
+    <row r="25" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A25" s="2">
+        <v>22</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="7"/>
+      <c r="J25" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="K25" s="2"/>
+      <c r="L25" s="2"/>
+    </row>
+    <row r="26" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="A26" s="2">
+        <v>23</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="7"/>
+      <c r="J26" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="K26" s="2"/>
+      <c r="L26" s="2"/>
+    </row>
+    <row r="27" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A27" s="2">
+        <v>24</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="7"/>
+      <c r="J27" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="K27" s="2"/>
+      <c r="L27" s="2"/>
+    </row>
+    <row r="28" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A28" s="2">
+        <v>25</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+      <c r="I28" s="7"/>
+      <c r="J28" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="K28" s="2"/>
+      <c r="L28" s="2"/>
+    </row>
+    <row r="29" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="2">
+        <v>26</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="I29" s="7"/>
+      <c r="J29" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="K29" s="2"/>
+      <c r="L29" s="2"/>
+    </row>
+    <row r="30" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="2">
+        <v>27</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="7"/>
+      <c r="J30" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="K30" s="2"/>
+      <c r="L30" s="2"/>
+    </row>
+    <row r="31" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="2">
+        <v>28</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="7"/>
+      <c r="J31" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="K31" s="2"/>
+      <c r="L31" s="2"/>
+    </row>
+    <row r="32" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A32" s="2">
+        <v>29</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="7"/>
+      <c r="J32" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="K32" s="2"/>
+      <c r="L32" s="2"/>
+    </row>
+    <row r="33" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <v>30</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+      <c r="I33" s="7"/>
+      <c r="J33" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="K33" s="2"/>
+      <c r="L33" s="2"/>
+    </row>
+    <row r="34" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="2">
+        <v>31</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+      <c r="I34" s="7"/>
+      <c r="J34" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="K34" s="2"/>
+      <c r="L34" s="2"/>
+    </row>
+    <row r="35" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A35" s="2">
+        <v>32</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="7"/>
+      <c r="J35" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="K35" s="2"/>
+      <c r="L35" s="2"/>
+    </row>
+    <row r="36" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A36" s="2">
+        <v>33</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="7"/>
+      <c r="J36" s="2"/>
+      <c r="K36" s="2"/>
+      <c r="L36" s="2"/>
+    </row>
+    <row r="37" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A37" s="2">
+        <v>34</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+      <c r="I37" s="7"/>
+      <c r="J37" s="2"/>
+      <c r="K37" s="2"/>
+      <c r="L37" s="2"/>
+    </row>
+    <row r="38" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A38" s="2">
+        <v>35</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
+      <c r="I38" s="7"/>
+      <c r="J38" s="2"/>
+      <c r="K38" s="2"/>
+      <c r="L38" s="2"/>
+    </row>
+    <row r="39" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A39" s="2">
+        <v>36</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+      <c r="I39" s="7"/>
+      <c r="J39" s="2"/>
+      <c r="K39" s="2"/>
+      <c r="L39" s="2"/>
+    </row>
+    <row r="40" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A40" s="2">
+        <v>37</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
+      <c r="I40" s="7"/>
+      <c r="J40" s="2"/>
+      <c r="K40" s="2"/>
+      <c r="L40" s="2"/>
+    </row>
+    <row r="41" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A41" s="2">
+        <v>38</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
+      <c r="I41" s="7"/>
+      <c r="J41" s="2"/>
+      <c r="K41" s="2"/>
+      <c r="L41" s="2"/>
+    </row>
+    <row r="42" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A42" s="2">
+        <v>39</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
+      <c r="I42" s="7"/>
+      <c r="J42" s="2"/>
+      <c r="K42" s="2"/>
+      <c r="L42" s="2"/>
+    </row>
+    <row r="43" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A43" s="2">
+        <v>40</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
+      <c r="I43" s="7"/>
+      <c r="J43" s="2"/>
+      <c r="K43" s="2"/>
+      <c r="L43" s="2"/>
+    </row>
+    <row r="44" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A44" s="2">
+        <v>41</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
+      <c r="H44" s="2"/>
+      <c r="I44" s="7"/>
+      <c r="J44" s="2"/>
+      <c r="K44" s="2"/>
+      <c r="L44" s="2"/>
+    </row>
+    <row r="45" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A45" s="2">
+        <v>42</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+      <c r="H45" s="2"/>
+      <c r="I45" s="7"/>
+      <c r="J45" s="2"/>
+      <c r="K45" s="2"/>
+      <c r="L45" s="2"/>
+    </row>
+    <row r="46" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A46" s="2">
+        <v>43</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2"/>
+      <c r="G46" s="2"/>
+      <c r="H46" s="2"/>
+      <c r="I46" s="7"/>
+      <c r="J46" s="2"/>
+      <c r="K46" s="2"/>
+      <c r="L46" s="2"/>
+    </row>
+    <row r="47" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A47" s="2">
+        <v>44</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
+      <c r="H47" s="2"/>
+      <c r="I47" s="7"/>
+      <c r="J47" s="2"/>
+      <c r="K47" s="2"/>
+      <c r="L47" s="2"/>
+    </row>
+    <row r="48" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A48" s="2">
+        <v>45</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="2"/>
+      <c r="G48" s="2"/>
+      <c r="H48" s="2"/>
+      <c r="I48" s="7"/>
+      <c r="J48" s="2"/>
+      <c r="K48" s="2"/>
+      <c r="L48" s="2"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <conditionalFormatting sqref="I4:I48">
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>$I4="FAIL"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="2">
+      <formula>$I4="PASS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4:I48" xr:uid="{9B456021-722F-45A6-B4AB-4D7CB37ED02F}">
+      <formula1>"PASS, FAIL"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B96F994C-1060-4B45-911D-957EF7B58CF0}">
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.28515625" customWidth="1"/>
     <col min="3" max="3" width="29.28515625" customWidth="1"/>
-    <col min="4" max="4" width="26" customWidth="1"/>
-    <col min="5" max="5" width="17.85546875" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="4" max="4" width="38.28515625" customWidth="1"/>
+    <col min="5" max="5" width="23.7109375" customWidth="1"/>
+    <col min="6" max="6" width="26.28515625" customWidth="1"/>
     <col min="8" max="8" width="10.5703125" customWidth="1"/>
     <col min="9" max="9" width="9.7109375" customWidth="1"/>
   </cols>
@@ -1798,7 +3469,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
@@ -1806,20 +3477,22 @@
         <v>10</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="F4" s="2"/>
+        <v>194</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>195</v>
+      </c>
       <c r="G4" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
+        <v>67</v>
+      </c>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
     </row>
     <row r="5" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
@@ -1829,20 +3502,24 @@
         <v>22</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
+        <v>110</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>196</v>
+      </c>
       <c r="G5" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-    </row>
-    <row r="6" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+    </row>
+    <row r="6" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>13</v>
       </c>
@@ -1850,20 +3527,24 @@
         <v>31</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
+        <v>122</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>197</v>
+      </c>
       <c r="G6" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-    </row>
-    <row r="7" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+    </row>
+    <row r="7" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>14</v>
       </c>
@@ -1871,20 +3552,24 @@
         <v>32</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
+        <v>121</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>198</v>
+      </c>
       <c r="G7" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-    </row>
-    <row r="8" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+    </row>
+    <row r="8" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>15</v>
       </c>
@@ -1892,20 +3577,24 @@
         <v>30</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
+        <v>120</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>199</v>
+      </c>
       <c r="G8" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-    </row>
-    <row r="9" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+    </row>
+    <row r="9" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>16</v>
       </c>
@@ -1913,20 +3602,24 @@
         <v>23</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
+        <v>119</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>200</v>
+      </c>
       <c r="G9" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-    </row>
-    <row r="10" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+    </row>
+    <row r="10" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>17</v>
       </c>
@@ -1934,20 +3627,24 @@
         <v>33</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
+        <v>118</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>205</v>
+      </c>
       <c r="G10" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-    </row>
-    <row r="11" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+    </row>
+    <row r="11" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>18</v>
       </c>
@@ -1955,20 +3652,24 @@
         <v>34</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
+        <v>117</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>201</v>
+      </c>
       <c r="G11" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-    </row>
-    <row r="12" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+    </row>
+    <row r="12" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>19</v>
       </c>
@@ -1976,20 +3677,24 @@
         <v>35</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
+        <v>116</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>206</v>
+      </c>
       <c r="G12" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-    </row>
-    <row r="13" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
+    </row>
+    <row r="13" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>20</v>
       </c>
@@ -1997,20 +3702,24 @@
         <v>36</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
+        <v>115</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>202</v>
+      </c>
       <c r="G13" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-    </row>
-    <row r="14" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+    </row>
+    <row r="14" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>21</v>
       </c>
@@ -2018,20 +3727,24 @@
         <v>37</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
+        <v>114</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>203</v>
+      </c>
       <c r="G14" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-    </row>
-    <row r="15" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+    </row>
+    <row r="15" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>24</v>
       </c>
@@ -2039,18 +3752,22 @@
         <v>38</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>204</v>
+      </c>
       <c r="G15" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
+        <v>67</v>
+      </c>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
     </row>
     <row r="16" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
@@ -2060,20 +3777,24 @@
         <v>39</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
+        <v>123</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>207</v>
+      </c>
       <c r="G16" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-    </row>
-    <row r="17" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+    </row>
+    <row r="17" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>26</v>
       </c>
@@ -2081,20 +3802,26 @@
         <v>40</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
+        <v>124</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>208</v>
+      </c>
       <c r="G17" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-    </row>
-    <row r="18" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="I17" s="9"/>
+    </row>
+    <row r="18" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>27</v>
       </c>
@@ -2102,18 +3829,22 @@
         <v>41</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
+        <v>125</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>209</v>
+      </c>
       <c r="G18" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
+        <v>67</v>
+      </c>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
     </row>
     <row r="19" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
@@ -2123,125 +3854,161 @@
         <v>42</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
+        <v>126</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>210</v>
+      </c>
       <c r="G19" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-    </row>
-    <row r="20" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+    </row>
+    <row r="20" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>29</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
+        <v>127</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>213</v>
+      </c>
       <c r="G20" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-    </row>
-    <row r="21" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="I20" s="9" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>45</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
+        <v>128</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>215</v>
+      </c>
       <c r="G21" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-    </row>
-    <row r="22" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+    </row>
+    <row r="22" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>46</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
+        <v>129</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>215</v>
+      </c>
       <c r="G22" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-    </row>
-    <row r="23" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+    </row>
+    <row r="23" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>47</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
+        <v>130</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>217</v>
+      </c>
       <c r="G23" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-    </row>
-    <row r="24" spans="1:9" ht="240" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="I23" s="9" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>48</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
+        <v>131</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>219</v>
+      </c>
       <c r="G24" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-    </row>
-    <row r="25" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="I24" s="9" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>49</v>
       </c>
@@ -2249,20 +4016,24 @@
         <v>54</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
+        <v>112</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>221</v>
+      </c>
       <c r="G25" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-    </row>
-    <row r="26" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H25" s="9"/>
+      <c r="I25" s="9"/>
+    </row>
+    <row r="26" spans="1:9" ht="195" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>50</v>
       </c>
@@ -2270,20 +4041,24 @@
         <v>55</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
+        <v>132</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>222</v>
+      </c>
       <c r="G26" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-    </row>
-    <row r="27" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
+    </row>
+    <row r="27" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>51</v>
       </c>
@@ -2291,83 +4066,101 @@
         <v>56</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
+        <v>133</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>224</v>
+      </c>
       <c r="G27" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-    </row>
-    <row r="28" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H27" s="9"/>
+      <c r="I27" s="9"/>
+    </row>
+    <row r="28" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>52</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>135</v>
+        <v>44</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
+        <v>134</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>225</v>
+      </c>
       <c r="G28" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-    </row>
-    <row r="29" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="I28" s="9"/>
+    </row>
+    <row r="29" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>61</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>136</v>
+        <v>53</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
+        <v>135</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>195</v>
+      </c>
       <c r="G29" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-    </row>
-    <row r="30" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H29" s="9"/>
+      <c r="I29" s="9"/>
+    </row>
+    <row r="30" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>62</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
+        <v>136</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>195</v>
+      </c>
       <c r="G30" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-    </row>
-    <row r="31" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="H30" s="9"/>
+      <c r="I30" s="9"/>
+    </row>
+    <row r="31" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>63</v>
       </c>
@@ -2375,20 +4168,28 @@
         <v>57</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
+        <v>137</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>226</v>
+      </c>
       <c r="G31" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
-    </row>
-    <row r="32" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="I31" s="9" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>64</v>
       </c>
@@ -2396,165 +4197,407 @@
         <v>58</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
+        <v>138</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>226</v>
+      </c>
       <c r="G32" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
-    </row>
-    <row r="33" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+      <c r="H32" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="I32" s="9" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>59</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
+        <v>139</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>226</v>
+      </c>
       <c r="G33" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-    </row>
-    <row r="34" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+      <c r="H33" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="I33" s="9" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>60</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
+        <v>140</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>226</v>
+      </c>
       <c r="G34" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
-    </row>
-    <row r="35" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+      <c r="H34" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="I34" s="9" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>65</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D35" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="G35" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H35" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="I35" s="9" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="180" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H35" s="2"/>
-      <c r="I35" s="2"/>
-    </row>
-    <row r="36" spans="1:9" ht="210" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
+      <c r="E36" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H36" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="I36" s="9" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="135" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B37" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="C37" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="G37" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="H37" s="9"/>
+      <c r="I37" s="9"/>
+    </row>
+    <row r="38" spans="1:9" ht="165" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="B38" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="H38" s="9"/>
+      <c r="I38" s="9"/>
+    </row>
+    <row r="39" spans="1:9" ht="165" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="7"/>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
-    </row>
-    <row r="37" spans="1:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="B37" s="2" t="s">
+      <c r="B39" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="7"/>
-      <c r="H37" s="2"/>
-      <c r="I37" s="2"/>
-    </row>
-    <row r="38" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
+      <c r="C39" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="H39" s="9"/>
+      <c r="I39" s="9"/>
+    </row>
+    <row r="40" spans="1:9" ht="120" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B40" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D40" s="8">
+        <v>39974</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="H40" s="9"/>
+      <c r="I40" s="9"/>
+    </row>
+    <row r="41" spans="1:9" ht="120" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D41" s="8">
+        <v>39609</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="H41" s="9"/>
+      <c r="I41" s="9"/>
+    </row>
+    <row r="42" spans="1:9" ht="120" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="7"/>
-      <c r="H38" s="2"/>
-      <c r="I38" s="2"/>
-    </row>
-    <row r="39" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="B39" s="2" t="s">
+      <c r="B42" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D42" s="8">
+        <v>18789</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="G42" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="H42" s="9"/>
+      <c r="I42" s="9"/>
+    </row>
+    <row r="43" spans="1:9" ht="120" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="7"/>
-      <c r="H39" s="2"/>
-      <c r="I39" s="2"/>
+      <c r="B43" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D43" s="8">
+        <v>18424</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="G43" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H43" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="I43" s="9" t="s">
+        <v>212</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="G4:G39">
-    <cfRule type="expression" dxfId="5" priority="1">
+  <conditionalFormatting sqref="G4:G43">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>$G4="FAIL"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>$G4="PASS"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4:G39" xr:uid="{82D003DA-E2AC-4A21-B01A-723544129566}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4:G43" xr:uid="{82D003DA-E2AC-4A21-B01A-723544129566}">
       <formula1>"PASS, FAIL"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C90AFD66-A454-40A3-926A-721D95719A41}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="1.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="24" x14ac:dyDescent="0.4">
+      <c r="A1" s="10" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="B3" t="s">
+        <v>243</v>
+      </c>
+      <c r="C3" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="B4" t="s">
+        <v>243</v>
+      </c>
+      <c r="C4">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="B5" t="s">
+        <v>245</v>
+      </c>
+      <c r="C5">
+        <f>COUNTIF(Table1[Status], "PASS")</f>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>241</v>
+      </c>
+      <c r="B6" t="s">
+        <v>245</v>
+      </c>
+      <c r="C6">
+        <f>COUNTIF(Table1[Status], "FAIL")</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
+        <v>242</v>
+      </c>
+      <c r="B7" t="s">
+        <v>245</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>